<commit_message>
made some graphs to highlight differences between composite vs efa scoring
</commit_message>
<xml_diff>
--- a/18_composite_workbook/Composite_Workbook.xlsx
+++ b/18_composite_workbook/Composite_Workbook.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="360">
   <si>
     <t xml:space="preserve">participant_id</t>
   </si>
@@ -83,11 +83,13 @@
   </si>
   <si>
     <t xml:space="preserve">I thought this was a boring activity.
-IMI Q3</t>
+IMI Q3
+(reverse scored: 8 - raw score; IMI uses 1-7, so min + max = 8)</t>
   </si>
   <si>
     <t xml:space="preserve">This activity did not hold my attention at all.
-IMI Q4</t>
+IMI Q4
+(reverse scored: 8 - raw score; IMI uses 1-7, so min + max = 8)</t>
   </si>
   <si>
     <t xml:space="preserve">I would describe this activity as very interesting.
@@ -107,7 +109,8 @@
   </si>
   <si>
     <t xml:space="preserve">I didn't try very hard to do well at this activity.
-IMI Q15</t>
+IMI Q15
+(reverse scored: 8 - raw score; IMI uses 1-7, so min + max = 8)</t>
   </si>
   <si>
     <t xml:space="preserve">I tried very hard on this activity.
@@ -119,7 +122,8 @@
   </si>
   <si>
     <t xml:space="preserve">I didn't put much energy into this.
-IMI Q18</t>
+IMI Q18
+(reverse scored: 8 - raw score; IMI uses 1-7, so min + max = 8)</t>
   </si>
   <si>
     <t xml:space="preserve">I think I am pretty good at this activity.
@@ -295,19 +299,23 @@
   </si>
   <si>
     <t xml:space="preserve">Using generative AI technologies such as ChatGPT to complete assignments undermines the value of a university education.
-BeliefsAboutAI Q17</t>
+BeliefsAboutAI Q17
+(reverse scored upstream as 6 - raw score because Beliefs uses 1-5 and min + max = 6)</t>
   </si>
   <si>
     <t xml:space="preserve">Generative AI technologies such as ChatGPT will limit my opportunities to interact with others and socialize while completing coursework.
-BeliefsAboutAI Q18</t>
+BeliefsAboutAI Q18
+(reverse scored upstream as 6 - raw score because Beliefs uses 1-5 and min + max = 6)</t>
   </si>
   <si>
     <t xml:space="preserve">Generative AI technologies such as ChatGPT will hinder my development of generic or transferable skills such as teamwork, problem-solving, and leadership skills.
-BeliefsAboutAI Q19</t>
+BeliefsAboutAI Q19
+(reverse scored upstream as 6 - raw score because Beliefs uses 1-5 and min + max = 6)</t>
   </si>
   <si>
     <t xml:space="preserve">I can become over-reliant on generative AI technologies.
-BeliefsAboutAI Q20</t>
+BeliefsAboutAI Q20
+(reverse scored upstream as 6 - raw score because Beliefs uses 1-5 and min + max = 6)</t>
   </si>
   <si>
     <t xml:space="preserve">051eD8</t>
@@ -683,6 +691,9 @@
   </si>
   <si>
     <t xml:space="preserve">I thought this was a boring activity.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shown on scored item scale used for composite averaging; reverse scored: 8 - raw score; IMI uses 1-7, so min + max = 8.</t>
   </si>
   <si>
     <t xml:space="preserve">IMI_Q4</t>
@@ -20827,7 +20838,7 @@
         <v>195</v>
       </c>
       <c r="K7" s="25" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
     </row>
     <row r="8">
@@ -20835,7 +20846,7 @@
         <v>188</v>
       </c>
       <c r="B8" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C8" s="25" t="s">
         <v>15</v>
@@ -20859,10 +20870,10 @@
         <v>4</v>
       </c>
       <c r="J8" s="25" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K8" s="25" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
     </row>
     <row r="9">
@@ -20870,7 +20881,7 @@
         <v>188</v>
       </c>
       <c r="B9" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C9" s="25" t="s">
         <v>16</v>
@@ -20894,7 +20905,7 @@
         <v>5</v>
       </c>
       <c r="J9" s="25" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="K9" s="25" t="s">
         <v>191</v>
@@ -20905,7 +20916,7 @@
         <v>188</v>
       </c>
       <c r="B10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C10" s="25" t="s">
         <v>17</v>
@@ -20929,7 +20940,7 @@
         <v>6</v>
       </c>
       <c r="J10" s="25" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="K10" s="25" t="s">
         <v>191</v>
@@ -20940,7 +20951,7 @@
         <v>188</v>
       </c>
       <c r="B11" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C11" s="25" t="s">
         <v>18</v>
@@ -20964,7 +20975,7 @@
         <v>7</v>
       </c>
       <c r="J11" s="25" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="K11" s="25" t="s">
         <v>191</v>
@@ -20975,7 +20986,7 @@
         <v>188</v>
       </c>
       <c r="B12" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C12" s="25" t="s">
         <v>19</v>
@@ -20999,7 +21010,7 @@
         <v>14</v>
       </c>
       <c r="J12" s="25" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="K12" s="25" t="s">
         <v>191</v>
@@ -21010,7 +21021,7 @@
         <v>188</v>
       </c>
       <c r="B13" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C13" s="25" t="s">
         <v>20</v>
@@ -21034,10 +21045,10 @@
         <v>15</v>
       </c>
       <c r="J13" s="25" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="K13" s="25" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
     </row>
     <row r="14">
@@ -21045,7 +21056,7 @@
         <v>188</v>
       </c>
       <c r="B14" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C14" s="25" t="s">
         <v>21</v>
@@ -21069,7 +21080,7 @@
         <v>16</v>
       </c>
       <c r="J14" s="25" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K14" s="25" t="s">
         <v>191</v>
@@ -21080,7 +21091,7 @@
         <v>188</v>
       </c>
       <c r="B15" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C15" s="25" t="s">
         <v>22</v>
@@ -21104,7 +21115,7 @@
         <v>17</v>
       </c>
       <c r="J15" s="25" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K15" s="25" t="s">
         <v>191</v>
@@ -21115,7 +21126,7 @@
         <v>188</v>
       </c>
       <c r="B16" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C16" s="25" t="s">
         <v>23</v>
@@ -21139,10 +21150,10 @@
         <v>18</v>
       </c>
       <c r="J16" s="25" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="K16" s="25" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
     </row>
     <row r="17">
@@ -21150,7 +21161,7 @@
         <v>188</v>
       </c>
       <c r="B17" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C17" s="25" t="s">
         <v>24</v>
@@ -21174,7 +21185,7 @@
         <v>8</v>
       </c>
       <c r="J17" s="25" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="K17" s="25" t="s">
         <v>191</v>
@@ -21185,7 +21196,7 @@
         <v>188</v>
       </c>
       <c r="B18" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C18" s="25" t="s">
         <v>25</v>
@@ -21209,7 +21220,7 @@
         <v>9</v>
       </c>
       <c r="J18" s="25" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="K18" s="25" t="s">
         <v>191</v>
@@ -21220,7 +21231,7 @@
         <v>188</v>
       </c>
       <c r="B19" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C19" s="25" t="s">
         <v>26</v>
@@ -21244,7 +21255,7 @@
         <v>10</v>
       </c>
       <c r="J19" s="25" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="K19" s="25" t="s">
         <v>191</v>
@@ -21255,7 +21266,7 @@
         <v>188</v>
       </c>
       <c r="B20" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C20" s="25" t="s">
         <v>27</v>
@@ -21279,7 +21290,7 @@
         <v>11</v>
       </c>
       <c r="J20" s="25" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="K20" s="25" t="s">
         <v>191</v>
@@ -21290,7 +21301,7 @@
         <v>188</v>
       </c>
       <c r="B21" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C21" s="25" t="s">
         <v>28</v>
@@ -21314,7 +21325,7 @@
         <v>12</v>
       </c>
       <c r="J21" s="25" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="K21" s="25" t="s">
         <v>191</v>
@@ -21325,25 +21336,25 @@
         <v>173</v>
       </c>
       <c r="B22" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C22" s="25" t="s">
         <v>4</v>
       </c>
       <c r="D22" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="E22" t="s">
+        <v>227</v>
+      </c>
+      <c r="F22" t="s">
         <v>225</v>
       </c>
-      <c r="E22" t="s">
-        <v>226</v>
-      </c>
-      <c r="F22" t="s">
-        <v>224</v>
-      </c>
       <c r="G22" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="H22" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="I22"/>
       <c r="J22" s="25"/>
@@ -21356,25 +21367,25 @@
         <v>173</v>
       </c>
       <c r="B23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C23" s="25" t="s">
         <v>5</v>
       </c>
       <c r="D23" s="17" t="s">
+        <v>231</v>
+      </c>
+      <c r="E23" t="s">
+        <v>227</v>
+      </c>
+      <c r="F23" t="s">
         <v>230</v>
       </c>
-      <c r="E23" t="s">
-        <v>226</v>
-      </c>
-      <c r="F23" t="s">
-        <v>229</v>
-      </c>
       <c r="G23" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="H23" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="I23"/>
       <c r="J23" s="25"/>
@@ -21387,25 +21398,25 @@
         <v>173</v>
       </c>
       <c r="B24" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C24" s="25" t="s">
         <v>6</v>
       </c>
       <c r="D24" s="18" t="s">
+        <v>235</v>
+      </c>
+      <c r="E24" t="s">
+        <v>227</v>
+      </c>
+      <c r="F24" t="s">
         <v>234</v>
       </c>
-      <c r="E24" t="s">
-        <v>226</v>
-      </c>
-      <c r="F24" t="s">
-        <v>233</v>
-      </c>
       <c r="G24" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H24" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="I24"/>
       <c r="J24" s="25"/>
@@ -21418,34 +21429,34 @@
         <v>188</v>
       </c>
       <c r="B25" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C25" s="25" t="s">
         <v>29</v>
       </c>
       <c r="D25" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="E25" t="s">
+        <v>227</v>
+      </c>
+      <c r="F25" t="s">
         <v>225</v>
       </c>
-      <c r="E25" t="s">
-        <v>226</v>
-      </c>
-      <c r="F25" t="s">
-        <v>224</v>
-      </c>
       <c r="G25" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="H25" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="I25" t="n">
         <v>1</v>
       </c>
       <c r="J25" s="25" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="K25" s="25" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="26">
@@ -21453,34 +21464,34 @@
         <v>188</v>
       </c>
       <c r="B26" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C26" s="25" t="s">
         <v>30</v>
       </c>
       <c r="D26" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="E26" t="s">
+        <v>227</v>
+      </c>
+      <c r="F26" t="s">
         <v>225</v>
       </c>
-      <c r="E26" t="s">
-        <v>226</v>
-      </c>
-      <c r="F26" t="s">
-        <v>224</v>
-      </c>
       <c r="G26" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="H26" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="I26" t="n">
         <v>3</v>
       </c>
       <c r="J26" s="25" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="K26" s="25" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="27">
@@ -21488,34 +21499,34 @@
         <v>188</v>
       </c>
       <c r="B27" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C27" s="25" t="s">
         <v>31</v>
       </c>
       <c r="D27" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="E27" t="s">
+        <v>227</v>
+      </c>
+      <c r="F27" t="s">
         <v>225</v>
       </c>
-      <c r="E27" t="s">
-        <v>226</v>
-      </c>
-      <c r="F27" t="s">
-        <v>224</v>
-      </c>
       <c r="G27" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="H27" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="I27" t="n">
         <v>5</v>
       </c>
       <c r="J27" s="25" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="K27" s="25" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="28">
@@ -21523,34 +21534,34 @@
         <v>188</v>
       </c>
       <c r="B28" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C28" s="25" t="s">
         <v>32</v>
       </c>
       <c r="D28" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="E28" t="s">
+        <v>227</v>
+      </c>
+      <c r="F28" t="s">
         <v>225</v>
       </c>
-      <c r="E28" t="s">
-        <v>226</v>
-      </c>
-      <c r="F28" t="s">
-        <v>224</v>
-      </c>
       <c r="G28" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="H28" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="I28" t="n">
         <v>9</v>
       </c>
       <c r="J28" s="25" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K28" s="25" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="29">
@@ -21558,34 +21569,34 @@
         <v>188</v>
       </c>
       <c r="B29" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C29" s="25" t="s">
         <v>33</v>
       </c>
       <c r="D29" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="E29" t="s">
+        <v>227</v>
+      </c>
+      <c r="F29" t="s">
         <v>225</v>
       </c>
-      <c r="E29" t="s">
-        <v>226</v>
-      </c>
-      <c r="F29" t="s">
-        <v>224</v>
-      </c>
       <c r="G29" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="H29" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="I29" t="n">
         <v>11</v>
       </c>
       <c r="J29" s="25" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="K29" s="25" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="30">
@@ -21593,34 +21604,34 @@
         <v>188</v>
       </c>
       <c r="B30" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C30" s="25" t="s">
         <v>34</v>
       </c>
       <c r="D30" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="E30" t="s">
+        <v>227</v>
+      </c>
+      <c r="F30" t="s">
         <v>225</v>
       </c>
-      <c r="E30" t="s">
-        <v>226</v>
-      </c>
-      <c r="F30" t="s">
-        <v>224</v>
-      </c>
       <c r="G30" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="H30" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="I30" t="n">
         <v>12</v>
       </c>
       <c r="J30" s="25" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="K30" s="25" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="31">
@@ -21628,34 +21639,34 @@
         <v>188</v>
       </c>
       <c r="B31" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C31" s="25" t="s">
         <v>35</v>
       </c>
       <c r="D31" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="E31" t="s">
+        <v>227</v>
+      </c>
+      <c r="F31" t="s">
         <v>225</v>
       </c>
-      <c r="E31" t="s">
-        <v>226</v>
-      </c>
-      <c r="F31" t="s">
-        <v>224</v>
-      </c>
       <c r="G31" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="H31" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="I31" t="n">
         <v>18</v>
       </c>
       <c r="J31" s="25" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K31" s="25" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="32">
@@ -21663,34 +21674,34 @@
         <v>188</v>
       </c>
       <c r="B32" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C32" s="25" t="s">
         <v>36</v>
       </c>
       <c r="D32" s="17" t="s">
+        <v>231</v>
+      </c>
+      <c r="E32" t="s">
+        <v>227</v>
+      </c>
+      <c r="F32" t="s">
         <v>230</v>
       </c>
-      <c r="E32" t="s">
-        <v>226</v>
-      </c>
-      <c r="F32" t="s">
-        <v>229</v>
-      </c>
       <c r="G32" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="H32" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="I32" t="n">
         <v>8</v>
       </c>
       <c r="J32" s="25" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="K32" s="25" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="33">
@@ -21698,34 +21709,34 @@
         <v>188</v>
       </c>
       <c r="B33" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C33" s="25" t="s">
         <v>37</v>
       </c>
       <c r="D33" s="17" t="s">
+        <v>231</v>
+      </c>
+      <c r="E33" t="s">
+        <v>227</v>
+      </c>
+      <c r="F33" t="s">
         <v>230</v>
       </c>
-      <c r="E33" t="s">
-        <v>226</v>
-      </c>
-      <c r="F33" t="s">
-        <v>229</v>
-      </c>
       <c r="G33" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="H33" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="I33" t="n">
         <v>10</v>
       </c>
       <c r="J33" s="25" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="K33" s="25" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="34">
@@ -21733,34 +21744,34 @@
         <v>188</v>
       </c>
       <c r="B34" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C34" s="25" t="s">
         <v>38</v>
       </c>
       <c r="D34" s="17" t="s">
+        <v>231</v>
+      </c>
+      <c r="E34" t="s">
+        <v>227</v>
+      </c>
+      <c r="F34" t="s">
         <v>230</v>
       </c>
-      <c r="E34" t="s">
-        <v>226</v>
-      </c>
-      <c r="F34" t="s">
-        <v>229</v>
-      </c>
       <c r="G34" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="H34" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="I34" t="n">
         <v>14</v>
       </c>
       <c r="J34" s="25" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="K34" s="25" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="35">
@@ -21768,34 +21779,34 @@
         <v>188</v>
       </c>
       <c r="B35" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C35" s="25" t="s">
         <v>39</v>
       </c>
       <c r="D35" s="17" t="s">
+        <v>231</v>
+      </c>
+      <c r="E35" t="s">
+        <v>227</v>
+      </c>
+      <c r="F35" t="s">
         <v>230</v>
       </c>
-      <c r="E35" t="s">
-        <v>226</v>
-      </c>
-      <c r="F35" t="s">
-        <v>229</v>
-      </c>
       <c r="G35" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="H35" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="I35" t="n">
         <v>15</v>
       </c>
       <c r="J35" s="25" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K35" s="25" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="36">
@@ -21803,34 +21814,34 @@
         <v>188</v>
       </c>
       <c r="B36" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C36" s="25" t="s">
         <v>40</v>
       </c>
       <c r="D36" s="17" t="s">
+        <v>231</v>
+      </c>
+      <c r="E36" t="s">
+        <v>227</v>
+      </c>
+      <c r="F36" t="s">
         <v>230</v>
       </c>
-      <c r="E36" t="s">
-        <v>226</v>
-      </c>
-      <c r="F36" t="s">
-        <v>229</v>
-      </c>
       <c r="G36" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="H36" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="I36" t="n">
         <v>17</v>
       </c>
       <c r="J36" s="25" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="K36" s="25" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="37">
@@ -21838,34 +21849,34 @@
         <v>188</v>
       </c>
       <c r="B37" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C37" s="25" t="s">
         <v>41</v>
       </c>
       <c r="D37" s="18" t="s">
+        <v>235</v>
+      </c>
+      <c r="E37" t="s">
+        <v>227</v>
+      </c>
+      <c r="F37" t="s">
         <v>234</v>
       </c>
-      <c r="E37" t="s">
-        <v>226</v>
-      </c>
-      <c r="F37" t="s">
-        <v>233</v>
-      </c>
       <c r="G37" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H37" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="I37" t="n">
         <v>2</v>
       </c>
       <c r="J37" s="25" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="K37" s="25" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="38">
@@ -21873,34 +21884,34 @@
         <v>188</v>
       </c>
       <c r="B38" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C38" s="25" t="s">
         <v>42</v>
       </c>
       <c r="D38" s="18" t="s">
+        <v>235</v>
+      </c>
+      <c r="E38" t="s">
+        <v>227</v>
+      </c>
+      <c r="F38" t="s">
         <v>234</v>
       </c>
-      <c r="E38" t="s">
-        <v>226</v>
-      </c>
-      <c r="F38" t="s">
-        <v>233</v>
-      </c>
       <c r="G38" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H38" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="I38" t="n">
         <v>19</v>
       </c>
       <c r="J38" s="25" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="K38" s="25" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="39">
@@ -21908,34 +21919,34 @@
         <v>188</v>
       </c>
       <c r="B39" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C39" s="25" t="s">
         <v>43</v>
       </c>
       <c r="D39" s="18" t="s">
+        <v>235</v>
+      </c>
+      <c r="E39" t="s">
+        <v>227</v>
+      </c>
+      <c r="F39" t="s">
         <v>234</v>
       </c>
-      <c r="E39" t="s">
-        <v>226</v>
-      </c>
-      <c r="F39" t="s">
-        <v>233</v>
-      </c>
       <c r="G39" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H39" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="I39" t="n">
         <v>20</v>
       </c>
       <c r="J39" s="25" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K39" s="25" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="40">
@@ -21943,25 +21954,25 @@
         <v>173</v>
       </c>
       <c r="B40" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C40" s="25" t="s">
         <v>7</v>
       </c>
       <c r="D40" s="19" t="s">
+        <v>270</v>
+      </c>
+      <c r="E40" t="s">
+        <v>271</v>
+      </c>
+      <c r="F40" t="s">
         <v>269</v>
       </c>
-      <c r="E40" t="s">
-        <v>270</v>
-      </c>
-      <c r="F40" t="s">
-        <v>268</v>
-      </c>
       <c r="G40" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H40" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="I40"/>
       <c r="J40" s="25"/>
@@ -21974,25 +21985,25 @@
         <v>173</v>
       </c>
       <c r="B41" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C41" s="25" t="s">
         <v>8</v>
       </c>
       <c r="D41" s="20" t="s">
+        <v>275</v>
+      </c>
+      <c r="E41" t="s">
+        <v>271</v>
+      </c>
+      <c r="F41" t="s">
         <v>274</v>
       </c>
-      <c r="E41" t="s">
-        <v>270</v>
-      </c>
-      <c r="F41" t="s">
-        <v>273</v>
-      </c>
       <c r="G41" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="H41" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="I41"/>
       <c r="J41" s="25"/>
@@ -22005,31 +22016,31 @@
         <v>188</v>
       </c>
       <c r="B42" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C42" s="25" t="s">
         <v>44</v>
       </c>
       <c r="D42" s="19" t="s">
+        <v>270</v>
+      </c>
+      <c r="E42" t="s">
+        <v>271</v>
+      </c>
+      <c r="F42" t="s">
         <v>269</v>
       </c>
-      <c r="E42" t="s">
-        <v>270</v>
-      </c>
-      <c r="F42" t="s">
-        <v>268</v>
-      </c>
       <c r="G42" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H42" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="I42" t="n">
         <v>4</v>
       </c>
       <c r="J42" s="25" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="K42" s="25" t="s">
         <v>191</v>
@@ -22040,31 +22051,31 @@
         <v>188</v>
       </c>
       <c r="B43" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C43" s="25" t="s">
         <v>45</v>
       </c>
       <c r="D43" s="19" t="s">
+        <v>270</v>
+      </c>
+      <c r="E43" t="s">
+        <v>271</v>
+      </c>
+      <c r="F43" t="s">
         <v>269</v>
       </c>
-      <c r="E43" t="s">
-        <v>270</v>
-      </c>
-      <c r="F43" t="s">
-        <v>268</v>
-      </c>
       <c r="G43" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H43" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="I43" t="n">
         <v>6</v>
       </c>
       <c r="J43" s="25" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="K43" s="25" t="s">
         <v>191</v>
@@ -22075,31 +22086,31 @@
         <v>188</v>
       </c>
       <c r="B44" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C44" s="25" t="s">
         <v>46</v>
       </c>
       <c r="D44" s="19" t="s">
+        <v>270</v>
+      </c>
+      <c r="E44" t="s">
+        <v>271</v>
+      </c>
+      <c r="F44" t="s">
         <v>269</v>
       </c>
-      <c r="E44" t="s">
-        <v>270</v>
-      </c>
-      <c r="F44" t="s">
-        <v>268</v>
-      </c>
       <c r="G44" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H44" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="I44" t="n">
         <v>7</v>
       </c>
       <c r="J44" s="25" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="K44" s="25" t="s">
         <v>191</v>
@@ -22110,31 +22121,31 @@
         <v>188</v>
       </c>
       <c r="B45" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C45" s="25" t="s">
         <v>47</v>
       </c>
       <c r="D45" s="19" t="s">
+        <v>270</v>
+      </c>
+      <c r="E45" t="s">
+        <v>271</v>
+      </c>
+      <c r="F45" t="s">
         <v>269</v>
       </c>
-      <c r="E45" t="s">
-        <v>270</v>
-      </c>
-      <c r="F45" t="s">
-        <v>268</v>
-      </c>
       <c r="G45" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H45" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="I45" t="n">
         <v>9</v>
       </c>
       <c r="J45" s="25" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="K45" s="25" t="s">
         <v>191</v>
@@ -22145,31 +22156,31 @@
         <v>188</v>
       </c>
       <c r="B46" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C46" s="25" t="s">
         <v>48</v>
       </c>
       <c r="D46" s="19" t="s">
+        <v>270</v>
+      </c>
+      <c r="E46" t="s">
+        <v>271</v>
+      </c>
+      <c r="F46" t="s">
         <v>269</v>
       </c>
-      <c r="E46" t="s">
-        <v>270</v>
-      </c>
-      <c r="F46" t="s">
-        <v>268</v>
-      </c>
       <c r="G46" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H46" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="I46" t="n">
         <v>10</v>
       </c>
       <c r="J46" s="25" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="K46" s="25" t="s">
         <v>191</v>
@@ -22180,31 +22191,31 @@
         <v>188</v>
       </c>
       <c r="B47" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C47" s="25" t="s">
         <v>49</v>
       </c>
       <c r="D47" s="19" t="s">
+        <v>270</v>
+      </c>
+      <c r="E47" t="s">
+        <v>271</v>
+      </c>
+      <c r="F47" t="s">
         <v>269</v>
       </c>
-      <c r="E47" t="s">
-        <v>270</v>
-      </c>
-      <c r="F47" t="s">
-        <v>268</v>
-      </c>
       <c r="G47" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H47" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="I47" t="n">
         <v>11</v>
       </c>
       <c r="J47" s="25" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K47" s="25" t="s">
         <v>191</v>
@@ -22215,31 +22226,31 @@
         <v>188</v>
       </c>
       <c r="B48" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C48" s="25" t="s">
         <v>50</v>
       </c>
       <c r="D48" s="19" t="s">
+        <v>270</v>
+      </c>
+      <c r="E48" t="s">
+        <v>271</v>
+      </c>
+      <c r="F48" t="s">
         <v>269</v>
       </c>
-      <c r="E48" t="s">
-        <v>270</v>
-      </c>
-      <c r="F48" t="s">
-        <v>268</v>
-      </c>
       <c r="G48" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H48" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="I48" t="n">
         <v>12</v>
       </c>
       <c r="J48" s="25" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="K48" s="25" t="s">
         <v>191</v>
@@ -22250,31 +22261,31 @@
         <v>188</v>
       </c>
       <c r="B49" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C49" s="25" t="s">
         <v>51</v>
       </c>
       <c r="D49" s="20" t="s">
+        <v>275</v>
+      </c>
+      <c r="E49" t="s">
+        <v>271</v>
+      </c>
+      <c r="F49" t="s">
         <v>274</v>
       </c>
-      <c r="E49" t="s">
-        <v>270</v>
-      </c>
-      <c r="F49" t="s">
-        <v>273</v>
-      </c>
       <c r="G49" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="H49" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="I49" t="n">
         <v>1</v>
       </c>
       <c r="J49" s="25" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="K49" s="25" t="s">
         <v>191</v>
@@ -22285,31 +22296,31 @@
         <v>188</v>
       </c>
       <c r="B50" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C50" s="25" t="s">
         <v>52</v>
       </c>
       <c r="D50" s="20" t="s">
+        <v>275</v>
+      </c>
+      <c r="E50" t="s">
+        <v>271</v>
+      </c>
+      <c r="F50" t="s">
         <v>274</v>
       </c>
-      <c r="E50" t="s">
-        <v>270</v>
-      </c>
-      <c r="F50" t="s">
-        <v>273</v>
-      </c>
       <c r="G50" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="H50" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="I50" t="n">
         <v>2</v>
       </c>
       <c r="J50" s="25" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="K50" s="25" t="s">
         <v>191</v>
@@ -22320,31 +22331,31 @@
         <v>188</v>
       </c>
       <c r="B51" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C51" s="25" t="s">
         <v>53</v>
       </c>
       <c r="D51" s="20" t="s">
+        <v>275</v>
+      </c>
+      <c r="E51" t="s">
+        <v>271</v>
+      </c>
+      <c r="F51" t="s">
         <v>274</v>
       </c>
-      <c r="E51" t="s">
-        <v>270</v>
-      </c>
-      <c r="F51" t="s">
-        <v>273</v>
-      </c>
       <c r="G51" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="H51" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="I51" t="n">
         <v>3</v>
       </c>
       <c r="J51" s="25" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="K51" s="25" t="s">
         <v>191</v>
@@ -22355,30 +22366,30 @@
         <v>173</v>
       </c>
       <c r="B52" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C52" s="25" t="s">
         <v>11</v>
       </c>
       <c r="D52" s="21" t="s">
+        <v>299</v>
+      </c>
+      <c r="E52" t="s">
+        <v>300</v>
+      </c>
+      <c r="F52" t="s">
         <v>298</v>
       </c>
-      <c r="E52" t="s">
-        <v>299</v>
-      </c>
-      <c r="F52" t="s">
-        <v>297</v>
-      </c>
       <c r="G52" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="H52" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="I52"/>
       <c r="J52" s="25"/>
       <c r="K52" s="25" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="53">
@@ -22386,25 +22397,25 @@
         <v>173</v>
       </c>
       <c r="B53" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C53" s="25" t="s">
         <v>10</v>
       </c>
       <c r="D53" s="22" t="s">
+        <v>305</v>
+      </c>
+      <c r="E53" t="s">
+        <v>300</v>
+      </c>
+      <c r="F53" t="s">
         <v>304</v>
       </c>
-      <c r="E53" t="s">
-        <v>299</v>
-      </c>
-      <c r="F53" t="s">
-        <v>303</v>
-      </c>
       <c r="G53" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="H53" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="I53"/>
       <c r="J53" s="25"/>
@@ -22417,25 +22428,25 @@
         <v>173</v>
       </c>
       <c r="B54" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C54" s="25" t="s">
         <v>9</v>
       </c>
       <c r="D54" s="23" t="s">
+        <v>309</v>
+      </c>
+      <c r="E54" t="s">
+        <v>300</v>
+      </c>
+      <c r="F54" t="s">
         <v>308</v>
       </c>
-      <c r="E54" t="s">
-        <v>299</v>
-      </c>
-      <c r="F54" t="s">
-        <v>307</v>
-      </c>
       <c r="G54" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="H54" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="I54"/>
       <c r="J54" s="25"/>
@@ -22448,34 +22459,34 @@
         <v>188</v>
       </c>
       <c r="B55" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C55" s="25" t="s">
         <v>67</v>
       </c>
       <c r="D55" s="21" t="s">
+        <v>299</v>
+      </c>
+      <c r="E55" t="s">
+        <v>300</v>
+      </c>
+      <c r="F55" t="s">
         <v>298</v>
       </c>
-      <c r="E55" t="s">
-        <v>299</v>
-      </c>
-      <c r="F55" t="s">
-        <v>297</v>
-      </c>
       <c r="G55" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="H55" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="I55" t="n">
         <v>17</v>
       </c>
       <c r="J55" s="25" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="K55" s="25" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="56">
@@ -22483,34 +22494,34 @@
         <v>188</v>
       </c>
       <c r="B56" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C56" s="25" t="s">
         <v>68</v>
       </c>
       <c r="D56" s="21" t="s">
+        <v>299</v>
+      </c>
+      <c r="E56" t="s">
+        <v>300</v>
+      </c>
+      <c r="F56" t="s">
         <v>298</v>
       </c>
-      <c r="E56" t="s">
-        <v>299</v>
-      </c>
-      <c r="F56" t="s">
-        <v>297</v>
-      </c>
       <c r="G56" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="H56" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="I56" t="n">
         <v>18</v>
       </c>
       <c r="J56" s="25" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="K56" s="25" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="57">
@@ -22518,34 +22529,34 @@
         <v>188</v>
       </c>
       <c r="B57" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C57" s="25" t="s">
         <v>69</v>
       </c>
       <c r="D57" s="21" t="s">
+        <v>299</v>
+      </c>
+      <c r="E57" t="s">
+        <v>300</v>
+      </c>
+      <c r="F57" t="s">
         <v>298</v>
       </c>
-      <c r="E57" t="s">
-        <v>299</v>
-      </c>
-      <c r="F57" t="s">
-        <v>297</v>
-      </c>
       <c r="G57" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="H57" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="I57" t="n">
         <v>19</v>
       </c>
       <c r="J57" s="25" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="K57" s="25" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="58">
@@ -22553,34 +22564,34 @@
         <v>188</v>
       </c>
       <c r="B58" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C58" s="25" t="s">
         <v>70</v>
       </c>
       <c r="D58" s="21" t="s">
+        <v>299</v>
+      </c>
+      <c r="E58" t="s">
+        <v>300</v>
+      </c>
+      <c r="F58" t="s">
         <v>298</v>
       </c>
-      <c r="E58" t="s">
-        <v>299</v>
-      </c>
-      <c r="F58" t="s">
-        <v>297</v>
-      </c>
       <c r="G58" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="H58" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="I58" t="n">
         <v>20</v>
       </c>
       <c r="J58" s="25" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="K58" s="25" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="59">
@@ -22588,31 +22599,31 @@
         <v>188</v>
       </c>
       <c r="B59" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C59" s="25" t="s">
         <v>64</v>
       </c>
       <c r="D59" s="22" t="s">
+        <v>305</v>
+      </c>
+      <c r="E59" t="s">
+        <v>300</v>
+      </c>
+      <c r="F59" t="s">
         <v>304</v>
       </c>
-      <c r="E59" t="s">
-        <v>299</v>
-      </c>
-      <c r="F59" t="s">
-        <v>303</v>
-      </c>
       <c r="G59" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="H59" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="I59" t="n">
         <v>6</v>
       </c>
       <c r="J59" s="25" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="K59" s="25" t="s">
         <v>191</v>
@@ -22623,31 +22634,31 @@
         <v>188</v>
       </c>
       <c r="B60" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C60" s="25" t="s">
         <v>65</v>
       </c>
       <c r="D60" s="22" t="s">
+        <v>305</v>
+      </c>
+      <c r="E60" t="s">
+        <v>300</v>
+      </c>
+      <c r="F60" t="s">
         <v>304</v>
       </c>
-      <c r="E60" t="s">
-        <v>299</v>
-      </c>
-      <c r="F60" t="s">
-        <v>303</v>
-      </c>
       <c r="G60" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="H60" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="I60" t="n">
         <v>21</v>
       </c>
       <c r="J60" s="25" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="K60" s="25" t="s">
         <v>191</v>
@@ -22658,31 +22669,31 @@
         <v>188</v>
       </c>
       <c r="B61" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C61" s="25" t="s">
         <v>66</v>
       </c>
       <c r="D61" s="22" t="s">
+        <v>305</v>
+      </c>
+      <c r="E61" t="s">
+        <v>300</v>
+      </c>
+      <c r="F61" t="s">
         <v>304</v>
       </c>
-      <c r="E61" t="s">
-        <v>299</v>
-      </c>
-      <c r="F61" t="s">
-        <v>303</v>
-      </c>
       <c r="G61" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="H61" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="I61" t="n">
         <v>22</v>
       </c>
       <c r="J61" s="25" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="K61" s="25" t="s">
         <v>191</v>
@@ -22693,31 +22704,31 @@
         <v>188</v>
       </c>
       <c r="B62" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C62" s="25" t="s">
         <v>54</v>
       </c>
       <c r="D62" s="23" t="s">
+        <v>309</v>
+      </c>
+      <c r="E62" t="s">
+        <v>300</v>
+      </c>
+      <c r="F62" t="s">
         <v>308</v>
       </c>
-      <c r="E62" t="s">
-        <v>299</v>
-      </c>
-      <c r="F62" t="s">
-        <v>307</v>
-      </c>
       <c r="G62" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="H62" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="I62" t="n">
         <v>7</v>
       </c>
       <c r="J62" s="25" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="K62" s="25" t="s">
         <v>191</v>
@@ -22728,31 +22739,31 @@
         <v>188</v>
       </c>
       <c r="B63" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C63" s="25" t="s">
         <v>55</v>
       </c>
       <c r="D63" s="23" t="s">
+        <v>309</v>
+      </c>
+      <c r="E63" t="s">
+        <v>300</v>
+      </c>
+      <c r="F63" t="s">
         <v>308</v>
       </c>
-      <c r="E63" t="s">
-        <v>299</v>
-      </c>
-      <c r="F63" t="s">
-        <v>307</v>
-      </c>
       <c r="G63" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="H63" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="I63" t="n">
         <v>8</v>
       </c>
       <c r="J63" s="25" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="K63" s="25" t="s">
         <v>191</v>
@@ -22763,31 +22774,31 @@
         <v>188</v>
       </c>
       <c r="B64" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C64" s="25" t="s">
         <v>56</v>
       </c>
       <c r="D64" s="23" t="s">
+        <v>309</v>
+      </c>
+      <c r="E64" t="s">
+        <v>300</v>
+      </c>
+      <c r="F64" t="s">
         <v>308</v>
       </c>
-      <c r="E64" t="s">
-        <v>299</v>
-      </c>
-      <c r="F64" t="s">
-        <v>307</v>
-      </c>
       <c r="G64" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="H64" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="I64" t="n">
         <v>9</v>
       </c>
       <c r="J64" s="25" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="K64" s="25" t="s">
         <v>191</v>
@@ -22798,31 +22809,31 @@
         <v>188</v>
       </c>
       <c r="B65" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C65" s="25" t="s">
         <v>57</v>
       </c>
       <c r="D65" s="23" t="s">
+        <v>309</v>
+      </c>
+      <c r="E65" t="s">
+        <v>300</v>
+      </c>
+      <c r="F65" t="s">
         <v>308</v>
       </c>
-      <c r="E65" t="s">
-        <v>299</v>
-      </c>
-      <c r="F65" t="s">
-        <v>307</v>
-      </c>
       <c r="G65" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="H65" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="I65" t="n">
         <v>10</v>
       </c>
       <c r="J65" s="25" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="K65" s="25" t="s">
         <v>191</v>
@@ -22833,31 +22844,31 @@
         <v>188</v>
       </c>
       <c r="B66" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C66" s="25" t="s">
         <v>58</v>
       </c>
       <c r="D66" s="23" t="s">
+        <v>309</v>
+      </c>
+      <c r="E66" t="s">
+        <v>300</v>
+      </c>
+      <c r="F66" t="s">
         <v>308</v>
       </c>
-      <c r="E66" t="s">
-        <v>299</v>
-      </c>
-      <c r="F66" t="s">
-        <v>307</v>
-      </c>
       <c r="G66" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="H66" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="I66" t="n">
         <v>11</v>
       </c>
       <c r="J66" s="25" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K66" s="25" t="s">
         <v>191</v>
@@ -22868,31 +22879,31 @@
         <v>188</v>
       </c>
       <c r="B67" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C67" s="25" t="s">
         <v>59</v>
       </c>
       <c r="D67" s="23" t="s">
+        <v>309</v>
+      </c>
+      <c r="E67" t="s">
+        <v>300</v>
+      </c>
+      <c r="F67" t="s">
         <v>308</v>
       </c>
-      <c r="E67" t="s">
-        <v>299</v>
-      </c>
-      <c r="F67" t="s">
-        <v>307</v>
-      </c>
       <c r="G67" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="H67" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="I67" t="n">
         <v>12</v>
       </c>
       <c r="J67" s="25" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="K67" s="25" t="s">
         <v>191</v>
@@ -22903,31 +22914,31 @@
         <v>188</v>
       </c>
       <c r="B68" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C68" s="25" t="s">
         <v>60</v>
       </c>
       <c r="D68" s="23" t="s">
+        <v>309</v>
+      </c>
+      <c r="E68" t="s">
+        <v>300</v>
+      </c>
+      <c r="F68" t="s">
         <v>308</v>
       </c>
-      <c r="E68" t="s">
-        <v>299</v>
-      </c>
-      <c r="F68" t="s">
-        <v>307</v>
-      </c>
       <c r="G68" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="H68" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="I68" t="n">
         <v>13</v>
       </c>
       <c r="J68" s="25" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="K68" s="25" t="s">
         <v>191</v>
@@ -22938,31 +22949,31 @@
         <v>188</v>
       </c>
       <c r="B69" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C69" s="25" t="s">
         <v>61</v>
       </c>
       <c r="D69" s="23" t="s">
+        <v>309</v>
+      </c>
+      <c r="E69" t="s">
+        <v>300</v>
+      </c>
+      <c r="F69" t="s">
         <v>308</v>
       </c>
-      <c r="E69" t="s">
-        <v>299</v>
-      </c>
-      <c r="F69" t="s">
-        <v>307</v>
-      </c>
       <c r="G69" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="H69" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="I69" t="n">
         <v>14</v>
       </c>
       <c r="J69" s="25" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="K69" s="25" t="s">
         <v>191</v>
@@ -22973,31 +22984,31 @@
         <v>188</v>
       </c>
       <c r="B70" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C70" s="25" t="s">
         <v>62</v>
       </c>
       <c r="D70" s="23" t="s">
+        <v>309</v>
+      </c>
+      <c r="E70" t="s">
+        <v>300</v>
+      </c>
+      <c r="F70" t="s">
         <v>308</v>
       </c>
-      <c r="E70" t="s">
-        <v>299</v>
-      </c>
-      <c r="F70" t="s">
-        <v>307</v>
-      </c>
       <c r="G70" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="H70" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="I70" t="n">
         <v>15</v>
       </c>
       <c r="J70" s="25" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="K70" s="25" t="s">
         <v>191</v>
@@ -23008,31 +23019,31 @@
         <v>188</v>
       </c>
       <c r="B71" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C71" s="25" t="s">
         <v>63</v>
       </c>
       <c r="D71" s="23" t="s">
+        <v>309</v>
+      </c>
+      <c r="E71" t="s">
+        <v>300</v>
+      </c>
+      <c r="F71" t="s">
         <v>308</v>
       </c>
-      <c r="E71" t="s">
-        <v>299</v>
-      </c>
-      <c r="F71" t="s">
-        <v>307</v>
-      </c>
       <c r="G71" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="H71" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="I71" t="n">
         <v>16</v>
       </c>
       <c r="J71" s="25" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="K71" s="25" t="s">
         <v>191</v>
@@ -23072,34 +23083,34 @@
         <v>167</v>
       </c>
       <c r="C1" s="24" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D1" s="24" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E1" s="24" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F1" s="24" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="G1" s="24" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="H1" s="24" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="I1" s="24" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="J1" s="24" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="K1" s="24" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="L1" s="24" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="2">
@@ -23110,7 +23121,7 @@
         <v>174</v>
       </c>
       <c r="C2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -23148,7 +23159,7 @@
         <v>180</v>
       </c>
       <c r="C3" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D3" t="n">
         <v>2</v>
@@ -23186,7 +23197,7 @@
         <v>184</v>
       </c>
       <c r="C4" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D4" t="n">
         <v>3</v>
@@ -23218,22 +23229,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B5" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C5" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D5" t="n">
         <v>1</v>
       </c>
       <c r="E5" t="s">
+        <v>229</v>
+      </c>
+      <c r="F5" t="s">
         <v>228</v>
-      </c>
-      <c r="F5" t="s">
-        <v>227</v>
       </c>
       <c r="G5" t="n">
         <v>82</v>
@@ -23256,22 +23267,22 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B6" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C6" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D6" t="n">
         <v>2</v>
       </c>
       <c r="E6" t="s">
+        <v>233</v>
+      </c>
+      <c r="F6" t="s">
         <v>232</v>
-      </c>
-      <c r="F6" t="s">
-        <v>231</v>
       </c>
       <c r="G6" t="n">
         <v>82</v>
@@ -23294,22 +23305,22 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B7" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C7" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D7" t="n">
         <v>3</v>
       </c>
       <c r="E7" t="s">
+        <v>237</v>
+      </c>
+      <c r="F7" t="s">
         <v>236</v>
-      </c>
-      <c r="F7" t="s">
-        <v>235</v>
       </c>
       <c r="G7" t="n">
         <v>82</v>
@@ -23332,22 +23343,22 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B8" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C8" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
       </c>
       <c r="E8" t="s">
+        <v>273</v>
+      </c>
+      <c r="F8" t="s">
         <v>272</v>
-      </c>
-      <c r="F8" t="s">
-        <v>271</v>
       </c>
       <c r="G8" t="n">
         <v>82</v>
@@ -23370,22 +23381,22 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B9" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C9" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D9" t="n">
         <v>2</v>
       </c>
       <c r="E9" t="s">
+        <v>277</v>
+      </c>
+      <c r="F9" t="s">
         <v>276</v>
-      </c>
-      <c r="F9" t="s">
-        <v>275</v>
       </c>
       <c r="G9" t="n">
         <v>82</v>
@@ -23408,22 +23419,22 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B10" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
       </c>
       <c r="E10" t="s">
+        <v>311</v>
+      </c>
+      <c r="F10" t="s">
         <v>310</v>
-      </c>
-      <c r="F10" t="s">
-        <v>309</v>
       </c>
       <c r="G10" t="n">
         <v>91</v>
@@ -23446,22 +23457,22 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C11" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D11" t="n">
         <v>2</v>
       </c>
       <c r="E11" t="s">
+        <v>307</v>
+      </c>
+      <c r="F11" t="s">
         <v>306</v>
-      </c>
-      <c r="F11" t="s">
-        <v>305</v>
       </c>
       <c r="G11" t="n">
         <v>91</v>
@@ -23484,22 +23495,22 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B12" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C12" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D12" t="n">
         <v>3</v>
       </c>
       <c r="E12" t="s">
+        <v>302</v>
+      </c>
+      <c r="F12" t="s">
         <v>301</v>
-      </c>
-      <c r="F12" t="s">
-        <v>300</v>
       </c>
       <c r="G12" t="n">
         <v>91</v>

</xml_diff>